<commit_message>
Add source-to-target mapping template, IRI campaign tab, and updated docs
- Updated success_queries.xlsx to follow source_to_target_mapping template
  format with metadata table (Target Column | source table | source column/logic)
  on top of each tab, followed by organic and campaign success queries
- Added IRI (International Money Transfer) tab using DDWV01.EXT_CDS_CHNL_EVNT
  with ACTVY_TYP_CD = '031' filter for transaction detection
- Tabs renamed to {MNE}_Success format (VCN_Success through IRI_Success)
- Updated VVD data dictionary, success events schema, and artifacts guide
- Updated metric code registry with all 46 campaigns
- Added quick_search.ps1 single-file PowerShell search script
- Updated SAS search keyword mappings and pipeline scripts

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metadata/success_queries.xlsx
+++ b/metadata/success_queries.xlsx
@@ -7,13 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VCN" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VDA" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VDT" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VUI" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VUT" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VAW" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IRI" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VCN_Success" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VDA_Success" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VDT_Success" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VUI_Success" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VUT_Success" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VAW_Success" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IRI_Success" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34,7 +34,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <sz val="14"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -70,7 +70,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -78,14 +78,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -456,306 +463,439 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A47"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VCN - Card Acquisition Success</t>
+          <t>Target Column</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>source table</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>source column/logic</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Metric: Card Acquisition | Source: DDWV01.VISA_DR_CRD_DLY | Date Field: ISS_DT</t>
-        </is>
-      </c>
+          <t>clnt_no</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CLNT_NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>acct_no</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>ORGANIC SUCCESS (All Events)</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>PROC SQL;</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>event_mnemonic_cd</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>VCN</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>event_type_cd</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>CREATE TABLE work.organic_success AS</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>event_attributes</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>JSON(STS_CD, SRVC_ID)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>SELECT * FROM CONNECTION TO EDW (</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>event_dt</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ISS_DT</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>snap_dt</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;GENERATED&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    SELECT DISTINCT</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        CLNT_NO,</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ISS_DT  AS SUCCESS_DT</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>job_id</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>&lt;GENERATED&gt;</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    FROM DDWV01.VISA_DR_CRD_DLY</t>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Query:</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    WHERE STS_CD IN ('06','08')</t>
+          <t>ORGANIC SUCCESS (All Events)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND SRVC_ID = 36</t>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>PROC SQL;</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND ISS_DT IS NOT NULL</t>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND SNAP_DT = (SELECT MAX(SNAP_DT) FROM DDWV01.VISA_DR_CRD_DLY WHERE SNAP_DT &gt;= CURRENT_DATE - 7)</t>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>CREATE TABLE work.organic_success AS</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>SELECT * FROM CONNECTION TO EDW (</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>);</t>
-        </is>
-      </c>
+      <c r="A19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>DISCONNECT FROM EDW;</t>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    SELECT DISTINCT</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>QUIT;</t>
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        CLNT_NO,</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ISS_DT  AS SUCCESS_DT</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">    FROM DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    WHERE STS_CD IN ('06','08')</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND SRVC_ID = 36</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND ISS_DT IS NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND SNAP_DT = (SELECT MAX(SNAP_DT) FROM DDWV01.VISA_DR_CRD_DLY WHERE SNAP_DT &gt;= CURRENT_DATE - 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>);</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>DISCONNECT FROM EDW;</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>QUIT;</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
           <t>CAMPAIGN SUCCESS (Tactic-Linked)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>PROC SQL;</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>CREATE TABLE work.campaign_success AS</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>SELECT * FROM CONNECTION TO EDW (</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    SELECT DISTINCT</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        A.CLNT_NO,</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        A.ISS_DT            AS SUCCESS_DT,</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TACTIC_ID,</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TREATMT_STRT_DT,</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TREATMT_END_DT</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    FROM DDWV01.VISA_DR_CRD_DLY        AS A</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    INNER JOIN DG6V01.TACTIC_EVNT_IP_AR_HIST AS B</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        ON A.CLNT_NO = B.CLNT_NO</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    WHERE A.STS_CD IN ('06','08')</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.SRVC_ID = 36</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.ISS_DT IS NOT NULL</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.SNAP_DT = (SELECT MAX(SNAP_DT) FROM DDWV01.VISA_DR_CRD_DLY WHERE SNAP_DT &gt;= CURRENT_DATE - 7)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(B.TACTIC_ID, 8, 3) = 'VCN'</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.ISS_DT BETWEEN B.TREATMT_STRT_DT AND B.TREATMT_END_DT</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>);</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>DISCONNECT FROM EDW;</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>QUIT;</t>
         </is>
@@ -772,306 +912,439 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A47"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VDA - Card Acquisition Success</t>
+          <t>Target Column</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>source table</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>source column/logic</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Metric: Card Acquisition | Source: DDWV01.VISA_DR_CRD_DLY | Date Field: ISS_DT</t>
-        </is>
-      </c>
+          <t>clnt_no</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CLNT_NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>acct_no</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>ORGANIC SUCCESS (All Events)</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>PROC SQL;</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>event_mnemonic_cd</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>VDA</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>event_type_cd</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>CREATE TABLE work.organic_success AS</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>event_attributes</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>JSON(STS_CD, SRVC_ID)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>SELECT * FROM CONNECTION TO EDW (</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>event_dt</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ISS_DT</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>snap_dt</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;GENERATED&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    SELECT DISTINCT</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        CLNT_NO,</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ISS_DT  AS SUCCESS_DT</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>job_id</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>&lt;GENERATED&gt;</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    FROM DDWV01.VISA_DR_CRD_DLY</t>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Query:</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    WHERE STS_CD IN ('06','08')</t>
+          <t>ORGANIC SUCCESS (All Events)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND SRVC_ID = 36</t>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>PROC SQL;</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND ISS_DT IS NOT NULL</t>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND SNAP_DT = (SELECT MAX(SNAP_DT) FROM DDWV01.VISA_DR_CRD_DLY WHERE SNAP_DT &gt;= CURRENT_DATE - 7)</t>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>CREATE TABLE work.organic_success AS</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>SELECT * FROM CONNECTION TO EDW (</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>);</t>
-        </is>
-      </c>
+      <c r="A19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>DISCONNECT FROM EDW;</t>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    SELECT DISTINCT</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>QUIT;</t>
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        CLNT_NO,</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ISS_DT  AS SUCCESS_DT</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">    FROM DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    WHERE STS_CD IN ('06','08')</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND SRVC_ID = 36</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND ISS_DT IS NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND SNAP_DT = (SELECT MAX(SNAP_DT) FROM DDWV01.VISA_DR_CRD_DLY WHERE SNAP_DT &gt;= CURRENT_DATE - 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>);</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>DISCONNECT FROM EDW;</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>QUIT;</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
           <t>CAMPAIGN SUCCESS (Tactic-Linked)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>PROC SQL;</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>CREATE TABLE work.campaign_success AS</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>SELECT * FROM CONNECTION TO EDW (</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    SELECT DISTINCT</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        A.CLNT_NO,</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        A.ISS_DT            AS SUCCESS_DT,</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TACTIC_ID,</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TREATMT_STRT_DT,</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TREATMT_END_DT</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    FROM DDWV01.VISA_DR_CRD_DLY        AS A</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    INNER JOIN DG6V01.TACTIC_EVNT_IP_AR_HIST AS B</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        ON A.CLNT_NO = B.CLNT_NO</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    WHERE A.STS_CD IN ('06','08')</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.SRVC_ID = 36</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.ISS_DT IS NOT NULL</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.SNAP_DT = (SELECT MAX(SNAP_DT) FROM DDWV01.VISA_DR_CRD_DLY WHERE SNAP_DT &gt;= CURRENT_DATE - 7)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(B.TACTIC_ID, 8, 3) = 'VDA'</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.ISS_DT BETWEEN B.TREATMT_STRT_DT AND B.TREATMT_END_DT</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>);</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>DISCONNECT FROM EDW;</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>QUIT;</t>
         </is>
@@ -1088,306 +1361,439 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A47"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VDT - Card Activation Success</t>
+          <t>Target Column</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>source table</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>source column/logic</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Metric: Card Activation | Source: DDWV01.VISA_DR_CRD_DLY | Date Field: ACTV_DT</t>
-        </is>
-      </c>
+          <t>clnt_no</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CLNT_NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>acct_no</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>ORGANIC SUCCESS (All Events)</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>PROC SQL;</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>event_mnemonic_cd</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>VDT</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>event_type_cd</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>CREATE TABLE work.organic_success AS</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>event_attributes</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>JSON(STS_CD, SRVC_ID)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>SELECT * FROM CONNECTION TO EDW (</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>event_dt</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ACTV_DT</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>snap_dt</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;GENERATED&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    SELECT DISTINCT</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        CLNT_NO,</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ACTV_DT  AS SUCCESS_DT</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>job_id</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>&lt;GENERATED&gt;</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    FROM DDWV01.VISA_DR_CRD_DLY</t>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Query:</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    WHERE STS_CD IN ('06','08')</t>
+          <t>ORGANIC SUCCESS (All Events)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND SRVC_ID = 36</t>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>PROC SQL;</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND ISS_DT IS NOT NULL</t>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND SNAP_DT = (SELECT MAX(SNAP_DT) FROM DDWV01.VISA_DR_CRD_DLY WHERE SNAP_DT &gt;= CURRENT_DATE - 7)</t>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>CREATE TABLE work.organic_success AS</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>SELECT * FROM CONNECTION TO EDW (</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>);</t>
-        </is>
-      </c>
+      <c r="A19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>DISCONNECT FROM EDW;</t>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    SELECT DISTINCT</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>QUIT;</t>
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        CLNT_NO,</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ACTV_DT  AS SUCCESS_DT</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">    FROM DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    WHERE STS_CD IN ('06','08')</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND SRVC_ID = 36</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND ISS_DT IS NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND SNAP_DT = (SELECT MAX(SNAP_DT) FROM DDWV01.VISA_DR_CRD_DLY WHERE SNAP_DT &gt;= CURRENT_DATE - 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>);</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>DISCONNECT FROM EDW;</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>QUIT;</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
           <t>CAMPAIGN SUCCESS (Tactic-Linked)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>PROC SQL;</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>CREATE TABLE work.campaign_success AS</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>SELECT * FROM CONNECTION TO EDW (</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    SELECT DISTINCT</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        A.CLNT_NO,</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        A.ACTV_DT            AS SUCCESS_DT,</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TACTIC_ID,</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TREATMT_STRT_DT,</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TREATMT_END_DT</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    FROM DDWV01.VISA_DR_CRD_DLY        AS A</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    INNER JOIN DG6V01.TACTIC_EVNT_IP_AR_HIST AS B</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        ON A.CLNT_NO = B.CLNT_NO</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    WHERE A.STS_CD IN ('06','08')</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.SRVC_ID = 36</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.ISS_DT IS NOT NULL</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.SNAP_DT = (SELECT MAX(SNAP_DT) FROM DDWV01.VISA_DR_CRD_DLY WHERE SNAP_DT &gt;= CURRENT_DATE - 7)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(B.TACTIC_ID, 8, 3) = 'VDT'</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.ACTV_DT BETWEEN B.TREATMT_STRT_DT AND B.TREATMT_END_DT</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>);</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>DISCONNECT FROM EDW;</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>QUIT;</t>
         </is>
@@ -1404,306 +1810,439 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A47"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VUI - Card Usage Success</t>
+          <t>Target Column</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>source table</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>source column/logic</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Metric: Card Usage | Source: DDWV01.VISA_DR_CRD_DLY | Date Field: ACTV_DT</t>
-        </is>
-      </c>
+          <t>clnt_no</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CLNT_NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>acct_no</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>ORGANIC SUCCESS (All Events)</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>PROC SQL;</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>event_mnemonic_cd</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>VUI</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>event_type_cd</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>CREATE TABLE work.organic_success AS</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>event_attributes</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>JSON(STS_CD, SRVC_ID)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>SELECT * FROM CONNECTION TO EDW (</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>event_dt</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ACTV_DT</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>snap_dt</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;GENERATED&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    SELECT DISTINCT</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        CLNT_NO,</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ACTV_DT  AS SUCCESS_DT</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>job_id</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>&lt;GENERATED&gt;</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    FROM DDWV01.VISA_DR_CRD_DLY</t>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Query:</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    WHERE STS_CD IN ('06','08')</t>
+          <t>ORGANIC SUCCESS (All Events)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND SRVC_ID = 36</t>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>PROC SQL;</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND ISS_DT IS NOT NULL</t>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND SNAP_DT = (SELECT MAX(SNAP_DT) FROM DDWV01.VISA_DR_CRD_DLY WHERE SNAP_DT &gt;= CURRENT_DATE - 7)</t>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>CREATE TABLE work.organic_success AS</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>SELECT * FROM CONNECTION TO EDW (</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>);</t>
-        </is>
-      </c>
+      <c r="A19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>DISCONNECT FROM EDW;</t>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    SELECT DISTINCT</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>QUIT;</t>
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        CLNT_NO,</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ACTV_DT  AS SUCCESS_DT</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">    FROM DDWV01.VISA_DR_CRD_DLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    WHERE STS_CD IN ('06','08')</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND SRVC_ID = 36</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND ISS_DT IS NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND SNAP_DT = (SELECT MAX(SNAP_DT) FROM DDWV01.VISA_DR_CRD_DLY WHERE SNAP_DT &gt;= CURRENT_DATE - 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>);</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>DISCONNECT FROM EDW;</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>QUIT;</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
           <t>CAMPAIGN SUCCESS (Tactic-Linked)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>PROC SQL;</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>CREATE TABLE work.campaign_success AS</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>SELECT * FROM CONNECTION TO EDW (</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    SELECT DISTINCT</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        A.CLNT_NO,</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        A.ACTV_DT            AS SUCCESS_DT,</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TACTIC_ID,</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TREATMT_STRT_DT,</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TREATMT_END_DT</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    FROM DDWV01.VISA_DR_CRD_DLY        AS A</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    INNER JOIN DG6V01.TACTIC_EVNT_IP_AR_HIST AS B</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        ON A.CLNT_NO = B.CLNT_NO</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    WHERE A.STS_CD IN ('06','08')</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.SRVC_ID = 36</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.ISS_DT IS NOT NULL</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.SNAP_DT = (SELECT MAX(SNAP_DT) FROM DDWV01.VISA_DR_CRD_DLY WHERE SNAP_DT &gt;= CURRENT_DATE - 7)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(B.TACTIC_ID, 8, 3) = 'VUI'</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.ACTV_DT BETWEEN B.TREATMT_STRT_DT AND B.TREATMT_END_DT</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>);</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>DISCONNECT FROM EDW;</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>QUIT;</t>
         </is>
@@ -1720,376 +2259,513 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A57"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VUT - Wallet Provisioning Success</t>
+          <t>Target Column</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>source table</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>source column/logic</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Metric: Wallet Provisioning | Source: DDWV05.CLNT_CRD_POS_LOG + DL_DECMAN.TOKEN_LIST | Date Field: TXN_DT</t>
+          <t>clnt_no</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>DDWV05.CLNT_CRD_POS_LOG</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CAST(SUBSTR(CLNT_CRD_NO, 7, 9) AS INTEGER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>acct_no</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>DDWV05.CLNT_CRD_POS_LOG</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>CLNT_CRD_NO</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>ORGANIC SUCCESS (All Events)</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>PROC SQL;</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>event_mnemonic_cd</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>VUT</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>event_type_cd</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>CREATE TABLE work.organic_success AS</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>event_attributes</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>DDWV05.CLNT_CRD_POS_LOG + DL_DECMAN.TOKEN_LIST</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>JSON(TOKN_REQSTR_ID, TOKEN_WALLET_IND)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>SELECT * FROM CONNECTION TO EDW (</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>event_dt</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>DDWV05.CLNT_CRD_POS_LOG</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>TXN_DT</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>snap_dt</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;GENERATED&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    SELECT DISTINCT</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        CAST(SUBSTR(B.CLNT_CRD_NO, 7, 9) AS INTEGER)  AS CLNT_NO,</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        B.TXN_DT                                        AS SUCCESS_DT</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>job_id</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>&lt;GENERATED&gt;</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    FROM DDWV05.CLNT_CRD_POS_LOG  AS B</t>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Query:</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>ORGANIC SUCCESS (All Events)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>PROC SQL;</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>CREATE TABLE work.organic_success AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>SELECT * FROM CONNECTION TO EDW (</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    SELECT DISTINCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        CAST(SUBSTR(B.CLNT_CRD_NO, 7, 9) AS INTEGER)  AS CLNT_NO,</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        B.TXN_DT                                        AS SUCCESS_DT</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    FROM DDWV05.CLNT_CRD_POS_LOG  AS B</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">    INNER JOIN DL_DECMAN.TOKEN_LIST AS C</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        ON B.TOKN_REQSTR_ID = C.TOKEN_ID</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    WHERE B.AMT1 = 0</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(B.CLNT_CRD_NO, 1, 5)  = '45190'</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND SUBSTR(B.VISA_DR_CRD_NO, 1, 5) = '45199'</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND SUBSTR(B.TOKN_REQSTR_ID, 1, 1) &gt; '0'</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND B.POS_ENTR_MODE_CD_NON_EMV = '000'</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND B.SRVC_CD = 36</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND C.TOKEN_WALLET_IND = 'Y'</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>);</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>DISCONNECT FROM EDW;</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>QUIT;</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">      AND SUBSTR(B.VISA_DR_CRD_NO, 1, 5) = '45199'</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND SUBSTR(B.TOKN_REQSTR_ID, 1, 1) &gt; '0'</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND B.POS_ENTR_MODE_CD_NON_EMV = '000'</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND B.SRVC_CD = 36</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND C.TOKEN_WALLET_IND = 'Y'</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>);</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>DISCONNECT FROM EDW;</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>QUIT;</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
           <t>CAMPAIGN SUCCESS (Tactic-Linked)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>PROC SQL;</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>CREATE TABLE work.campaign_success AS</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>SELECT * FROM CONNECTION TO EDW (</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    SELECT DISTINCT</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        CAST(SUBSTR(B.CLNT_CRD_NO, 7, 9) AS INTEGER)  AS CLNT_NO,</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TXN_DT                                        AS SUCCESS_DT,</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        D.TACTIC_ID,</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        D.TREATMT_STRT_DT,</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        D.TREATMT_END_DT</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    FROM DDWV05.CLNT_CRD_POS_LOG  AS B</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    INNER JOIN DL_DECMAN.TOKEN_LIST AS C</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        ON B.TOKN_REQSTR_ID = C.TOKEN_ID</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    INNER JOIN DG6V01.TACTIC_EVNT_IP_AR_HIST AS D</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        ON CAST(SUBSTR(B.CLNT_CRD_NO, 7, 9) AS INTEGER) = D.CLNT_NO</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    WHERE B.AMT1 = 0</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(B.CLNT_CRD_NO, 1, 5)  = '45190'</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(B.VISA_DR_CRD_NO, 1, 5) = '45199'</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(B.TOKN_REQSTR_ID, 1, 1) &gt; '0'</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND B.POS_ENTR_MODE_CD_NON_EMV = '000'</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND B.SRVC_CD = 36</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND C.TOKEN_WALLET_IND = 'Y'</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(D.TACTIC_ID, 8, 3) = 'VUT'</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND B.TXN_DT BETWEEN D.TREATMT_STRT_DT AND D.TREATMT_END_DT</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>);</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>DISCONNECT FROM EDW;</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>QUIT;</t>
         </is>
@@ -2106,376 +2782,513 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A57"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VAW - Wallet Provisioning Success</t>
+          <t>Target Column</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>source table</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>source column/logic</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Metric: Wallet Provisioning | Source: DDWV05.CLNT_CRD_POS_LOG + DL_DECMAN.TOKEN_LIST | Date Field: TXN_DT</t>
+          <t>clnt_no</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>DDWV05.CLNT_CRD_POS_LOG</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CAST(SUBSTR(CLNT_CRD_NO, 7, 9) AS INTEGER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>acct_no</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>DDWV05.CLNT_CRD_POS_LOG</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>CLNT_CRD_NO</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>ORGANIC SUCCESS (All Events)</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>PROC SQL;</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>event_mnemonic_cd</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>VAW</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>event_type_cd</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>CREATE TABLE work.organic_success AS</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>event_attributes</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>DDWV05.CLNT_CRD_POS_LOG + DL_DECMAN.TOKEN_LIST</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>JSON(TOKN_REQSTR_ID, TOKEN_WALLET_IND)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>SELECT * FROM CONNECTION TO EDW (</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>event_dt</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>DDWV05.CLNT_CRD_POS_LOG</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>TXN_DT</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>snap_dt</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;GENERATED&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    SELECT DISTINCT</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        CAST(SUBSTR(B.CLNT_CRD_NO, 7, 9) AS INTEGER)  AS CLNT_NO,</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        B.TXN_DT                                        AS SUCCESS_DT</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>job_id</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>&lt;GENERATED&gt;</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    FROM DDWV05.CLNT_CRD_POS_LOG  AS B</t>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Query:</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>ORGANIC SUCCESS (All Events)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>PROC SQL;</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>CREATE TABLE work.organic_success AS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>SELECT * FROM CONNECTION TO EDW (</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    SELECT DISTINCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        CAST(SUBSTR(B.CLNT_CRD_NO, 7, 9) AS INTEGER)  AS CLNT_NO,</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        B.TXN_DT                                        AS SUCCESS_DT</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    FROM DDWV05.CLNT_CRD_POS_LOG  AS B</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">    INNER JOIN DL_DECMAN.TOKEN_LIST AS C</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        ON B.TOKN_REQSTR_ID = C.TOKEN_ID</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    WHERE B.AMT1 = 0</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(B.CLNT_CRD_NO, 1, 5)  = '45190'</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND SUBSTR(B.VISA_DR_CRD_NO, 1, 5) = '45199'</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND SUBSTR(B.TOKN_REQSTR_ID, 1, 1) &gt; '0'</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND B.POS_ENTR_MODE_CD_NON_EMV = '000'</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND B.SRVC_CD = 36</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      AND C.TOKEN_WALLET_IND = 'Y'</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>);</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>DISCONNECT FROM EDW;</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>QUIT;</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">      AND SUBSTR(B.VISA_DR_CRD_NO, 1, 5) = '45199'</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND SUBSTR(B.TOKN_REQSTR_ID, 1, 1) &gt; '0'</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND B.POS_ENTR_MODE_CD_NON_EMV = '000'</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND B.SRVC_CD = 36</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      AND C.TOKEN_WALLET_IND = 'Y'</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>);</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>DISCONNECT FROM EDW;</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>QUIT;</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
           <t>CAMPAIGN SUCCESS (Tactic-Linked)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>PROC SQL;</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>CREATE TABLE work.campaign_success AS</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>SELECT * FROM CONNECTION TO EDW (</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    SELECT DISTINCT</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        CAST(SUBSTR(B.CLNT_CRD_NO, 7, 9) AS INTEGER)  AS CLNT_NO,</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TXN_DT                                        AS SUCCESS_DT,</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        D.TACTIC_ID,</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        D.TREATMT_STRT_DT,</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        D.TREATMT_END_DT</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    FROM DDWV05.CLNT_CRD_POS_LOG  AS B</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    INNER JOIN DL_DECMAN.TOKEN_LIST AS C</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        ON B.TOKN_REQSTR_ID = C.TOKEN_ID</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    INNER JOIN DG6V01.TACTIC_EVNT_IP_AR_HIST AS D</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        ON CAST(SUBSTR(B.CLNT_CRD_NO, 7, 9) AS INTEGER) = D.CLNT_NO</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    WHERE B.AMT1 = 0</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(B.CLNT_CRD_NO, 1, 5)  = '45190'</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(B.VISA_DR_CRD_NO, 1, 5) = '45199'</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(B.TOKN_REQSTR_ID, 1, 1) &gt; '0'</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND B.POS_ENTR_MODE_CD_NON_EMV = '000'</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND B.SRVC_CD = 36</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND C.TOKEN_WALLET_IND = 'Y'</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(D.TACTIC_ID, 8, 3) = 'VAW'</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND B.TXN_DT BETWEEN D.TREATMT_STRT_DT AND D.TREATMT_END_DT</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>);</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>DISCONNECT FROM EDW;</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>QUIT;</t>
         </is>
@@ -2492,264 +3305,409 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>IRI - International Money Transfer Success</t>
+          <t>Target Column</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>source table</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>source column/logic</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Metric: IMT Transaction | Source: DDWV01.EXT_CDS_CHNL_EVNT | Date Field: CAPTR_DT | Filter: ACTVY_TYP_CD = '031'</t>
+          <t>clnt_no</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.EXT_CDS_CHNL_EVNT</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CLNT_NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>acct_no</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.EXT_CDS_CHNL_EVNT</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>AR_ID</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>ORGANIC SUCCESS (All Events)</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.EXT_CDS_CHNL_EVNT</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>EVNT_AMT_CAD</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>PROC SQL;</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>event_mnemonic_cd</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>IRI</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>event_type_cd</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>CREATE TABLE work.organic_success AS</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>event_attributes</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.EXT_CDS_CHNL_EVNT</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>JSON(CHNL_TYP_CD, EVNT_CRNCY_CD, ACTVY_TYP_CD)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>SELECT * FROM CONNECTION TO EDW (</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>event_dt</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>DDWV01.EXT_CDS_CHNL_EVNT</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>CAPTR_DT</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>snap_dt</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;GENERATED&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    SELECT DISTINCT</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        CLNT_NO,</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        CAPTR_DT  AS SUCCESS_DT</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>job_id</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>&lt;GENERATED&gt;</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    FROM DDWV01.EXT_CDS_CHNL_EVNT</t>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Query:</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    WHERE ACTVY_TYP_CD = '031'        /* 031 = International Money Transfer */</t>
+          <t>ORGANIC SUCCESS (All Events)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr"/>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>PROC SQL;</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>);</t>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>DISCONNECT FROM EDW;</t>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>CREATE TABLE work.organic_success AS</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>QUIT;</t>
-        </is>
-      </c>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>SELECT * FROM CONNECTION TO EDW (</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">    SELECT DISTINCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        CLNT_NO,</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        CAPTR_DT  AS SUCCESS_DT</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    FROM DDWV01.EXT_CDS_CHNL_EVNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    WHERE ACTVY_TYP_CD = '031'        /* 031 = International Money Transfer */</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>);</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>DISCONNECT FROM EDW;</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>QUIT;</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
           <t>CAMPAIGN SUCCESS (Tactic-Linked)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>PROC SQL;</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>CONNECT TO TERADATA AS EDW (MODE=TERADATA);</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>CREATE TABLE work.campaign_success AS</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>SELECT * FROM CONNECTION TO EDW (</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    SELECT DISTINCT</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        A.CLNT_NO,</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        A.CAPTR_DT           AS SUCCESS_DT,</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TACTIC_ID,</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TREATMT_STRT_DT,</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        B.TREATMT_END_DT</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    FROM DDWV01.EXT_CDS_CHNL_EVNT        AS A</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    INNER JOIN DG6V01.TACTIC_EVNT_IP_AR_HIST AS B</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">        ON A.CLNT_NO = B.CLNT_NO</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    WHERE A.ACTVY_TYP_CD = '031'          /* 031 = International Money Transfer */</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND SUBSTR(B.TACTIC_ID, 8, 3) = 'IRI'</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">      AND A.CAPTR_DT BETWEEN B.TREATMT_STRT_DT AND B.TREATMT_END_DT</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>);</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>DISCONNECT FROM EDW;</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>QUIT;</t>
         </is>

</xml_diff>